<commit_message>
feat: apply three approved ingredient terminology decisions
</commit_message>
<xml_diff>
--- a/docs/INGREDIENT_TERMINOLOGY_REVIEW.xlsx
+++ b/docs/INGREDIENT_TERMINOLOGY_REVIEW.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terim incelemesi" sheetId="1" r:id="R15e973b3d08a4cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terim incelemesi" sheetId="1" r:id="R00e76ae3fcc24025"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -237,7 +237,7 @@
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Malzeme ID"/>
     <x:tableColumn id="2" name="Sabit anahtar"/>
-    <x:tableColumn id="3" name="Türkçe ad"/>
+    <x:tableColumn id="3" name="Önceki Türkçe ad"/>
     <x:tableColumn id="4" name="İngilizce ad"/>
     <x:tableColumn id="5" name="Diğer adlar"/>
     <x:tableColumn id="6" name="Kategoriler"/>
@@ -246,7 +246,7 @@
     <x:tableColumn id="9" name="Kanıt bağlantıları"/>
     <x:tableColumn id="10" name="Güven ve gerekçe"/>
     <x:tableColumn id="11" name="Durum"/>
-    <x:tableColumn id="12" name="İnsan kararı"/>
+    <x:tableColumn id="12" name="İnsan kararı / yeni ad"/>
     <x:tableColumn id="13" name="İnceleyen / tarih"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -474,7 +474,7 @@
         <x:v>Sabit anahtar</x:v>
       </x:c>
       <x:c r="C1" s="10" t="str">
-        <x:v>Türkçe ad</x:v>
+        <x:v>Önceki Türkçe ad</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
         <x:v>İngilizce ad</x:v>
@@ -501,7 +501,7 @@
         <x:v>Durum</x:v>
       </x:c>
       <x:c r="L1" s="10" t="str">
-        <x:v>İnsan kararı</x:v>
+        <x:v>İnsan kararı / yeni ad</x:v>
       </x:c>
       <x:c r="M1" s="11" t="str">
         <x:v>İnceleyen / tarih</x:v>
@@ -646,9 +646,11 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L5" s="14" t="str"/>
+        <x:v>Kullanıcı kararı uygulandı</x:v>
+      </x:c>
+      <x:c r="L5" s="14" t="str">
+        <x:v>Frenk kimyonu tohumu</x:v>
+      </x:c>
       <x:c r="M5" s="15" t="str"/>
     </x:row>
     <x:row r="6" ht="80" customHeight="1">
@@ -753,9 +755,11 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K8" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L8" s="14" t="str"/>
+        <x:v>Kullanıcı kararı uygulandı</x:v>
+      </x:c>
+      <x:c r="L8" s="14" t="str">
+        <x:v>Tam tahıllı mavi mısır unu</x:v>
+      </x:c>
       <x:c r="M8" s="15" t="str"/>
     </x:row>
     <x:row r="9" ht="80" customHeight="1">
@@ -788,9 +792,11 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K9" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L9" s="14" t="str"/>
+        <x:v>Kullanıcı kararı uygulandı</x:v>
+      </x:c>
+      <x:c r="L9" s="14" t="str">
+        <x:v>Badem püresi (sade, tuz ilavesiz)</x:v>
+      </x:c>
       <x:c r="M9" s="15" t="str"/>
     </x:row>
     <x:row r="10" ht="80" customHeight="1">
@@ -1150,7 +1156,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce3dc205e64e46d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f87bbb2b4bc4444"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: release final reviewed ingredient terminology decisions
</commit_message>
<xml_diff>
--- a/docs/INGREDIENT_TERMINOLOGY_REVIEW.xlsx
+++ b/docs/INGREDIENT_TERMINOLOGY_REVIEW.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terim incelemesi" sheetId="1" r:id="R00e76ae3fcc24025"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Terim incelemesi" sheetId="1" r:id="R882b3ab5c1934711"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -232,13 +232,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TerminologyReview" displayName="TerminologyReview" ref="A1:M19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M19"/>
-  <x:tableColumns count="13">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TerminologyReview" displayName="TerminologyReview" ref="A1:O19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:O19"/>
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="Malzeme ID"/>
     <x:tableColumn id="2" name="Sabit anahtar"/>
     <x:tableColumn id="3" name="Önceki Türkçe ad"/>
-    <x:tableColumn id="4" name="İngilizce ad"/>
+    <x:tableColumn id="4" name="Önceki İngilizce ad"/>
     <x:tableColumn id="5" name="Diğer adlar"/>
     <x:tableColumn id="6" name="Kategoriler"/>
     <x:tableColumn id="7" name="İnceleme nedeni"/>
@@ -246,8 +246,10 @@
     <x:tableColumn id="9" name="Kanıt bağlantıları"/>
     <x:tableColumn id="10" name="Güven ve gerekçe"/>
     <x:tableColumn id="11" name="Durum"/>
-    <x:tableColumn id="12" name="İnsan kararı / yeni ad"/>
-    <x:tableColumn id="13" name="İnceleyen / tarih"/>
+    <x:tableColumn id="12" name="Karar kodu"/>
+    <x:tableColumn id="13" name="Seçilen Türkçe ad"/>
+    <x:tableColumn id="14" name="Seçilen İngilizce ad"/>
+    <x:tableColumn id="15" name="İnceleyen / tarih"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -461,9 +463,11 @@
     <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="70" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="54" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="26" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="27" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="36" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -477,7 +481,7 @@
         <x:v>Önceki Türkçe ad</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
-        <x:v>İngilizce ad</x:v>
+        <x:v>Önceki İngilizce ad</x:v>
       </x:c>
       <x:c r="E1" s="10" t="str">
         <x:v>Diğer adlar</x:v>
@@ -501,9 +505,15 @@
         <x:v>Durum</x:v>
       </x:c>
       <x:c r="L1" s="10" t="str">
-        <x:v>İnsan kararı / yeni ad</x:v>
-      </x:c>
-      <x:c r="M1" s="11" t="str">
+        <x:v>Karar kodu</x:v>
+      </x:c>
+      <x:c r="M1" s="10" t="str">
+        <x:v>Seçilen Türkçe ad</x:v>
+      </x:c>
+      <x:c r="N1" s="10" t="str">
+        <x:v>Seçilen İngilizce ad</x:v>
+      </x:c>
+      <x:c r="O1" s="11" t="str">
         <x:v>İnceleyen / tarih</x:v>
       </x:c>
     </x:row>
@@ -537,10 +547,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K2" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L2" s="14" t="str"/>
-      <x:c r="M2" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L2" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M2" s="14" t="str"/>
+      <x:c r="N2" s="14" t="str"/>
+      <x:c r="O2" s="15" t="str"/>
     </x:row>
     <x:row r="3" ht="80" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -574,10 +588,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K3" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L3" s="14" t="str"/>
-      <x:c r="M3" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L3" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M3" s="14" t="str"/>
+      <x:c r="N3" s="14" t="str"/>
+      <x:c r="O3" s="15" t="str"/>
     </x:row>
     <x:row r="4" ht="80" customHeight="1">
       <x:c r="A4" s="12" t="str">
@@ -609,10 +627,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K4" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L4" s="14" t="str"/>
-      <x:c r="M4" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L4" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M4" s="14" t="str"/>
+      <x:c r="N4" s="14" t="str"/>
+      <x:c r="O4" s="15" t="str"/>
     </x:row>
     <x:row r="5" ht="80" customHeight="1">
       <x:c r="A5" s="12" t="str">
@@ -646,12 +668,16 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K5" s="13" t="str">
-        <x:v>Kullanıcı kararı uygulandı</x:v>
-      </x:c>
-      <x:c r="L5" s="14" t="str">
+        <x:v>Kullanıcı adı uygulandı</x:v>
+      </x:c>
+      <x:c r="L5" s="13" t="str">
+        <x:v>user-approved-name</x:v>
+      </x:c>
+      <x:c r="M5" s="14" t="str">
         <x:v>Frenk kimyonu tohumu</x:v>
       </x:c>
-      <x:c r="M5" s="15" t="str"/>
+      <x:c r="N5" s="14" t="str"/>
+      <x:c r="O5" s="15" t="str"/>
     </x:row>
     <x:row r="6" ht="80" customHeight="1">
       <x:c r="A6" s="12" t="str">
@@ -683,10 +709,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K6" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L6" s="14" t="str"/>
-      <x:c r="M6" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L6" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M6" s="14" t="str"/>
+      <x:c r="N6" s="14" t="str"/>
+      <x:c r="O6" s="15" t="str"/>
     </x:row>
     <x:row r="7" ht="80" customHeight="1">
       <x:c r="A7" s="12" t="str">
@@ -718,10 +748,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K7" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L7" s="14" t="str"/>
-      <x:c r="M7" s="15" t="str"/>
+        <x:v>Ek doğrulama gerekli</x:v>
+      </x:c>
+      <x:c r="L7" s="13" t="str">
+        <x:v>retain-pending-human-review</x:v>
+      </x:c>
+      <x:c r="M7" s="14" t="str"/>
+      <x:c r="N7" s="14" t="str"/>
+      <x:c r="O7" s="15" t="str"/>
     </x:row>
     <x:row r="8" ht="80" customHeight="1">
       <x:c r="A8" s="12" t="str">
@@ -755,12 +789,16 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K8" s="13" t="str">
-        <x:v>Kullanıcı kararı uygulandı</x:v>
-      </x:c>
-      <x:c r="L8" s="14" t="str">
+        <x:v>Kullanıcı adı uygulandı</x:v>
+      </x:c>
+      <x:c r="L8" s="13" t="str">
+        <x:v>user-approved-name</x:v>
+      </x:c>
+      <x:c r="M8" s="14" t="str">
         <x:v>Tam tahıllı mavi mısır unu</x:v>
       </x:c>
-      <x:c r="M8" s="15" t="str"/>
+      <x:c r="N8" s="14" t="str"/>
+      <x:c r="O8" s="15" t="str"/>
     </x:row>
     <x:row r="9" ht="80" customHeight="1">
       <x:c r="A9" s="12" t="str">
@@ -792,12 +830,16 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K9" s="13" t="str">
-        <x:v>Kullanıcı kararı uygulandı</x:v>
-      </x:c>
-      <x:c r="L9" s="14" t="str">
+        <x:v>Kullanıcı adı uygulandı</x:v>
+      </x:c>
+      <x:c r="L9" s="13" t="str">
+        <x:v>user-approved-name</x:v>
+      </x:c>
+      <x:c r="M9" s="14" t="str">
         <x:v>Badem püresi (sade, tuz ilavesiz)</x:v>
       </x:c>
-      <x:c r="M9" s="15" t="str"/>
+      <x:c r="N9" s="14" t="str"/>
+      <x:c r="O9" s="15" t="str"/>
     </x:row>
     <x:row r="10" ht="80" customHeight="1">
       <x:c r="A10" s="12" t="str">
@@ -829,10 +871,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K10" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L10" s="14" t="str"/>
-      <x:c r="M10" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L10" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M10" s="14" t="str"/>
+      <x:c r="N10" s="14" t="str"/>
+      <x:c r="O10" s="15" t="str"/>
     </x:row>
     <x:row r="11" ht="80" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -864,10 +910,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K11" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L11" s="14" t="str"/>
-      <x:c r="M11" s="15" t="str"/>
+        <x:v>Ek doğrulama gerekli</x:v>
+      </x:c>
+      <x:c r="L11" s="13" t="str">
+        <x:v>retain-pending-human-review</x:v>
+      </x:c>
+      <x:c r="M11" s="14" t="str"/>
+      <x:c r="N11" s="14" t="str"/>
+      <x:c r="O11" s="15" t="str"/>
     </x:row>
     <x:row r="12" ht="80" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -899,10 +949,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K12" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L12" s="14" t="str"/>
-      <x:c r="M12" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L12" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str"/>
+      <x:c r="N12" s="14" t="str"/>
+      <x:c r="O12" s="15" t="str"/>
     </x:row>
     <x:row r="13" ht="80" customHeight="1">
       <x:c r="A13" s="12" t="str">
@@ -934,10 +988,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K13" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L13" s="14" t="str"/>
-      <x:c r="M13" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L13" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str"/>
+      <x:c r="N13" s="14" t="str"/>
+      <x:c r="O13" s="15" t="str"/>
     </x:row>
     <x:row r="14" ht="80" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -971,10 +1029,16 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K14" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L14" s="14" t="str"/>
-      <x:c r="M14" s="15" t="str"/>
+        <x:v>Kullanıcı adı uygulandı</x:v>
+      </x:c>
+      <x:c r="L14" s="13" t="str">
+        <x:v>user-approved-name</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>Club soda (kokteyl sodası)</x:v>
+      </x:c>
+      <x:c r="N14" s="14" t="str"/>
+      <x:c r="O14" s="15" t="str"/>
     </x:row>
     <x:row r="15" ht="80" customHeight="1">
       <x:c r="A15" s="12" t="str">
@@ -1006,10 +1070,16 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K15" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L15" s="14" t="str"/>
-      <x:c r="M15" s="15" t="str"/>
+        <x:v>Kullanıcı adı uygulandı</x:v>
+      </x:c>
+      <x:c r="L15" s="13" t="str">
+        <x:v>user-approved-name</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str"/>
+      <x:c r="N15" s="14" t="str">
+        <x:v>Einkorn wheat (siyez)</x:v>
+      </x:c>
+      <x:c r="O15" s="15" t="str"/>
     </x:row>
     <x:row r="16" ht="80" customHeight="1">
       <x:c r="A16" s="12" t="str">
@@ -1041,10 +1111,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K16" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L16" s="14" t="str"/>
-      <x:c r="M16" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L16" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str"/>
+      <x:c r="N16" s="14" t="str"/>
+      <x:c r="O16" s="15" t="str"/>
     </x:row>
     <x:row r="17" ht="80" customHeight="1">
       <x:c r="A17" s="12" t="str">
@@ -1076,10 +1150,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K17" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L17" s="14" t="str"/>
-      <x:c r="M17" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L17" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str"/>
+      <x:c r="N17" s="14" t="str"/>
+      <x:c r="O17" s="15" t="str"/>
     </x:row>
     <x:row r="18" ht="80" customHeight="1">
       <x:c r="A18" s="12" t="str">
@@ -1113,10 +1191,14 @@
         <x:v>moderate: Pinned source supports the English identity/form. Independent Turkish culinary terminology approval is absent.</x:v>
       </x:c>
       <x:c r="K18" s="13" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L18" s="14" t="str"/>
-      <x:c r="M18" s="15" t="str"/>
+        <x:v>Ad korundu (kullanıcı kararı)</x:v>
+      </x:c>
+      <x:c r="L18" s="13" t="str">
+        <x:v>user-authorized-retain-name</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str"/>
+      <x:c r="N18" s="14" t="str"/>
+      <x:c r="O18" s="15" t="str"/>
     </x:row>
     <x:row r="19" ht="80" customHeight="1">
       <x:c r="A19" s="16" t="str">
@@ -1148,15 +1230,19 @@
         <x:v>low: Source identity is pinned, but the preferred Turkish culinary term/form is not independently linguistically verified.</x:v>
       </x:c>
       <x:c r="K19" s="17" t="str">
-        <x:v>İnsan incelemesi bekliyor</x:v>
-      </x:c>
-      <x:c r="L19" s="18" t="str"/>
-      <x:c r="M19" s="19" t="str"/>
+        <x:v>Ek doğrulama gerekli</x:v>
+      </x:c>
+      <x:c r="L19" s="17" t="str">
+        <x:v>retain-pending-human-review</x:v>
+      </x:c>
+      <x:c r="M19" s="18" t="str"/>
+      <x:c r="N19" s="18" t="str"/>
+      <x:c r="O19" s="19" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f87bbb2b4bc4444"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R610fecd203cf427a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>